<commit_message>
tollTariff: entryTollLocationID instead of toTollLocationID
</commit_message>
<xml_diff>
--- a/FIRESTORE-Data-Pump/DATA_PUMP_IN.xlsx
+++ b/FIRESTORE-Data-Pump/DATA_PUMP_IN.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\#GitHubLocalRepository\#TollManagement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\#GitHubLocalRepository\#TollManagement\FIRESTORE-Data-Pump\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1E0082-7286-4236-BC2F-A7B2D0EF634D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52EBAADA-5763-4D21-A13C-616548D113DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D16E0085-8F60-4DBB-8D98-B35955C2B72A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D16E0085-8F60-4DBB-8D98-B35955C2B72A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$I$1:$L$30</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="203">
   <si>
     <t>VID00002</t>
   </si>
@@ -495,13 +496,166 @@
   </si>
   <si>
     <t>Vehicles with 3 Axles or more</t>
+  </si>
+  <si>
+    <t>boothID</t>
+  </si>
+  <si>
+    <t>laneCount</t>
+  </si>
+  <si>
+    <t>tollLocationID</t>
+  </si>
+  <si>
+    <t>BID00001</t>
+  </si>
+  <si>
+    <t>BID00002</t>
+  </si>
+  <si>
+    <t>BID00003</t>
+  </si>
+  <si>
+    <t>BID00004</t>
+  </si>
+  <si>
+    <t>BID00005</t>
+  </si>
+  <si>
+    <t>BID00006</t>
+  </si>
+  <si>
+    <t>BID00007</t>
+  </si>
+  <si>
+    <t>BID00008</t>
+  </si>
+  <si>
+    <t>BID00009</t>
+  </si>
+  <si>
+    <t>BID00010</t>
+  </si>
+  <si>
+    <t>BID00011</t>
+  </si>
+  <si>
+    <t>BID00012</t>
+  </si>
+  <si>
+    <t>BID00013</t>
+  </si>
+  <si>
+    <t>BID00014</t>
+  </si>
+  <si>
+    <t>BID00015</t>
+  </si>
+  <si>
+    <t>BID00016</t>
+  </si>
+  <si>
+    <t>BID00017</t>
+  </si>
+  <si>
+    <t>BID00018</t>
+  </si>
+  <si>
+    <t>BID00019</t>
+  </si>
+  <si>
+    <t>BID00020</t>
+  </si>
+  <si>
+    <t>BID00021</t>
+  </si>
+  <si>
+    <t>BID00022</t>
+  </si>
+  <si>
+    <t>BID00023</t>
+  </si>
+  <si>
+    <t>BID00024</t>
+  </si>
+  <si>
+    <t>BID00025</t>
+  </si>
+  <si>
+    <t>BID00026</t>
+  </si>
+  <si>
+    <t>BID00027</t>
+  </si>
+  <si>
+    <t>BID00028</t>
+  </si>
+  <si>
+    <t>BID00029</t>
+  </si>
+  <si>
+    <t>BID00030</t>
+  </si>
+  <si>
+    <t>BID00031</t>
+  </si>
+  <si>
+    <t>BID00032</t>
+  </si>
+  <si>
+    <t>BID00033</t>
+  </si>
+  <si>
+    <t>BID00034</t>
+  </si>
+  <si>
+    <t>BID00035</t>
+  </si>
+  <si>
+    <t>BID00036</t>
+  </si>
+  <si>
+    <t>BID00037</t>
+  </si>
+  <si>
+    <t>BID00038</t>
+  </si>
+  <si>
+    <t>BID00039</t>
+  </si>
+  <si>
+    <t>BID00040</t>
+  </si>
+  <si>
+    <t>BID00041</t>
+  </si>
+  <si>
+    <t>BID00042</t>
+  </si>
+  <si>
+    <t>BID00043</t>
+  </si>
+  <si>
+    <t>BID00044</t>
+  </si>
+  <si>
+    <t>BID00045</t>
+  </si>
+  <si>
+    <t>BID00046</t>
+  </si>
+  <si>
+    <t>BID00047</t>
+  </si>
+  <si>
+    <t>BID00048</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -540,6 +694,12 @@
       <color theme="1"/>
       <name val="Google Sans"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -561,7 +721,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -572,6 +732,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -931,7 +1092,7 @@
       </c>
       <c r="L2" s="1">
         <f ca="1">RAND()</f>
-        <v>0.35723648597803548</v>
+        <v>0.96635256817667059</v>
       </c>
     </row>
     <row r="3" spans="2:12">
@@ -2061,4 +2222,561 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5219AEBE-20EC-4248-BFA8-A258133FA43D}">
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="8">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" s="8">
+        <v>3</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="8">
+        <v>4</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="8">
+        <v>5</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" s="8">
+        <v>6</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="8">
+        <v>7</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="8">
+        <v>8</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="8">
+        <v>1</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="8">
+        <v>2</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="8">
+        <v>3</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="8">
+        <v>4</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="8">
+        <v>5</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15" s="8">
+        <v>6</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="8">
+        <v>7</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B17" s="8">
+        <v>8</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="8">
+        <v>9</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="8">
+        <v>10</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="8">
+        <v>1</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B21" s="8">
+        <v>2</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="8">
+        <v>3</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="8">
+        <v>4</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="8">
+        <v>5</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B25" s="8">
+        <v>6</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B26" s="8">
+        <v>7</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="B27" s="8">
+        <v>8</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B28" s="8">
+        <v>9</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B29" s="8">
+        <v>10</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" s="8">
+        <v>1</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B31" s="8">
+        <v>2</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B32" s="8">
+        <v>3</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B33" s="8">
+        <v>4</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B34" s="8">
+        <v>5</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="B35" s="8">
+        <v>6</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" s="8">
+        <v>7</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B37" s="8">
+        <v>8</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="B38" s="8">
+        <v>9</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="B39" s="8">
+        <v>10</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B40" s="8">
+        <v>1</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B41" s="8">
+        <v>2</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B42" s="8">
+        <v>3</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B43" s="8">
+        <v>4</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B44" s="8">
+        <v>5</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B45" s="8">
+        <v>6</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B46" s="8">
+        <v>7</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B47" s="8">
+        <v>8</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B48" s="8">
+        <v>9</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B49" s="8">
+        <v>10</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>